<commit_message>
docs: revise action plan priorities (token/MFA/tests/retention)
</commit_message>
<xml_diff>
--- a/Specs/Sara-Arch_Action_Plan.xlsx
+++ b/Specs/Sara-Arch_Action_Plan.xlsx
@@ -8,11 +8,12 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 - Immediate" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 - Short Term" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 3 - Medium Term" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 4 - Long Term" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Results" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do Now (24h)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 - This Week" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 - Short Term" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 3 - Medium Term" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 4 - Long Term" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Results" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -604,7 +605,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Owner GitHub 2FA disabled + exposed GitHub token still active</t>
+          <t>Exposed active GitHub OAuth token + owner GitHub 2FA disabled</t>
         </is>
       </c>
     </row>
@@ -625,7 +626,7 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Manual hardening (MFA, 2FA, branch protection, restore testing) and several business UI modules are still pending.</t>
+          <t>The highest-priority risks are active account-security issues (exposed token, disabled 2FA/MFA) and financial-calculation correctness (supervision, balance math, retention).</t>
         </is>
       </c>
     </row>
@@ -653,22 +654,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="80" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="47" customWidth="1" min="5" max="5"/>
+    <col width="59" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Phase 1 — Immediate (this week)</t>
+          <t>Do Now — Next 24 hours</t>
         </is>
       </c>
     </row>
@@ -712,12 +713,12 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Run verify_high_priority.sql + tenant_isolation.sql + check Security Advisor UI</t>
+          <t>Revoke exposed GitHub OAuth token immediately</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -732,7 +733,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Zero high/medium Security Advisor warnings</t>
+          <t>Old token returns 401 / no longer listed in GitHub tokens</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -742,34 +743,34 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Manual Supabase step</t>
+          <t>Active incident; do not wait for a phase</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>0.2</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Insert Resend key + sender into app_settings and send test email</t>
+          <t>Enable GitHub 2FA on Gendy92 owner account</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Feature</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Test user receives new password email</t>
+          <t>2FA status enabled in GitHub settings</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -779,14 +780,14 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Use Supabase SQL Editor</t>
+          <t>Prevents account takeover</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -823,27 +824,27 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Enable GitHub 2FA on Gendy92 owner account</t>
+          <t>Insert Resend key + sender into app_settings and send test email</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>2FA status enabled in GitHub settings</t>
+          <t>Test user receives new password email</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -853,34 +854,34 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Prevents account takeover</t>
+          <t>Use Supabase SQL Editor</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Protect main (and dev.2) with required status checks</t>
+          <t>Run verify_high_priority.sql + tenant_isolation.sql + check Security Advisor UI</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>DevOps</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Cannot push directly; PRs require CI pass</t>
+          <t>Zero high/medium Security Advisor warnings</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -890,118 +891,7 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Branch protection rules</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>1.6</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Patch vitest/vite/esbuild vulnerabilities</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Quality</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>npm audit returns 0 high/critical</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>Dev-only but should be clean</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>1.7</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Fix ESLint warnings (npm run lint:fix + manual review)</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Quality</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>npm run lint shows 0 warnings</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>35 warnings currently</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>1.8</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Fast-forward or delete dev.2</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>DevOps</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>main and dev.2 are not diverged</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>dev.2 is 6 commits behind</t>
+          <t>Manual Supabase step</t>
         </is>
       </c>
     </row>
@@ -1019,22 +909,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="67" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="47" customWidth="1" min="5" max="5"/>
+    <col width="56" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="43" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Phase 2 — Short Term (next 2–4 weeks)</t>
+          <t>Phase 1 — This week</t>
         </is>
       </c>
     </row>
@@ -1078,17 +968,17 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Add Items catalog UI</t>
+          <t>Design decision: supervision system-locked audit row</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Architecture</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -1098,7 +988,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Screen lists/CRUD items table</t>
+          <t>Decision doc agreed; implementation ticket created</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -1108,24 +998,24 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Code exists, no UI</t>
+          <t>See docs/DECISION_supervision_audit_row.md</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Add Custody expenses UI</t>
+          <t>Design decision: retention / holdback model</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Architecture</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -1135,7 +1025,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Direct custody expense entry</t>
+          <t>Decision doc agreed; implementation ticket created</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -1145,24 +1035,24 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Currently tracked by returned_amount only</t>
+          <t>See docs/DECISION_retention_holdback.md</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Add Employee transactions UI</t>
+          <t>Add UI input validation to block paid_amount &gt; amount before save</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>UX/Quality</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -1172,7 +1062,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Add/edit advances, penalties, bonuses</t>
+          <t>Save button disabled / inline error when paid &gt; amount</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -1182,34 +1072,34 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Only consumed in payroll now</t>
+          <t>Do not rely only on server-side rejection</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Add Salary history UI</t>
+          <t>Add unit tests for balance, supervision, and payroll math</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Quality</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Screen shows employee_salary_history</t>
+          <t>Core calculation paths covered; CI green</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -1219,24 +1109,24 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Table exists, no UI</t>
+          <t>Silent financial bugs are client-facing errors</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Build real Settings page</t>
+          <t>Patch vitest/vite/esbuild vulnerabilities</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Quality</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -1246,7 +1136,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Configure currency, logo, default supervision</t>
+          <t>npm audit returns 0 high/critical</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -1256,34 +1146,34 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Currently placeholder</t>
+          <t>Dev-only but should be clean</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>2.6</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Implement restore-from-backup</t>
+          <t>Fix ESLint warnings (npm run lint:fix + manual review)</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Quality</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Upload ZIP/JSON and import tables</t>
+          <t>npm run lint shows 0 warnings</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -1293,24 +1183,24 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Backup is export-only</t>
+          <t>35 warnings currently</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>2.7</t>
+          <t>1.7</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Add server-side pagination + indexes</t>
+          <t>Protect main (and dev.2) with required status checks</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>DevOps</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -1320,7 +1210,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Large lists load &lt;1s</t>
+          <t>Cannot push directly; PRs require CI pass</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -1330,34 +1220,34 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>transactions, clients, vendors</t>
+          <t>Branch protection rules</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>2.8</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Update outdated docs (TEST_PLAN, TEST_DATA, APP_TABS_GUIDE, ROADMAP)</t>
+          <t>Fast-forward or delete dev.2</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>DevOps</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Docs match current runtime</t>
+          <t>main and dev.2 are not diverged</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -1367,118 +1257,7 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Target v83/v105 references</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>2.9</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Set up staging Supabase + monthly restore test</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>DevOps</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>Successful restore verified monthly</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>DR proof</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>2.10</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Revoke exposed GitHub OAuth token and rotate Supabase keys</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>Old token/key disabled, new in GitHub Secrets</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>User previously accepted risk</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>2.11</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Add unit tests for api.js, app-core.js, app-loaders.js, crud.js</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Quality</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>Coverage &gt;50% for core modules</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>Only 3 test files now</t>
+          <t>dev.2 is 6 commits behind</t>
         </is>
       </c>
     </row>
@@ -1491,6 +1270,520 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="63" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="43" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Phase 2 — Short Term (next 2–4 weeks)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Implement retention / holdback tracking</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Retention withheld/released per project; reports correct</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Often contractually required</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Generate system-locked supervision audit rows (if decided)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>System rows appear at period close; non-editable; tagged</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Depends on 1.1 decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Add Items catalog UI</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Screen lists/CRUD items table</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Code exists, no UI</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Add Custody expenses UI</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Direct custody expense entry</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Currently tracked by returned_amount only</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Add Employee transactions UI</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Add/edit advances, penalties, bonuses</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Only consumed in payroll now</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Add Salary history UI</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Screen shows employee_salary_history</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Table exists, no UI</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Build real Settings page</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Configure currency, logo, default supervision</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Currently placeholder</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>2.8</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Implement restore-from-backup</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Upload ZIP/JSON and import tables</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Backup is export-only</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>2.9</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Add server-side pagination + indexes</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Large lists load &lt;1s</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>transactions, clients, vendors</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>2.10</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Update outdated docs (TEST_PLAN, TEST_DATA, APP_TABS_GUIDE, ROADMAP)</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Docs match current runtime</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Target v83/v105 references</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>2.11</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Set up staging Supabase + monthly restore test</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>DevOps</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Successful restore verified monthly</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>DR proof</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>2.12</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Rotate Supabase service-role and anon keys</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>New keys in GitHub Secrets; old keys disabled after CI passes</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Periodic rotation</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1758,7 +2051,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1960,7 +2253,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
docs: update action plan for v294 retention/supervision implementation
</commit_message>
<xml_diff>
--- a/Specs/Sara-Arch_Action_Plan.xlsx
+++ b/Specs/Sara-Arch_Action_Plan.xlsx
@@ -617,7 +617,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>&gt; Live version: v292</t>
+          <t>&gt; Live version: v294</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>**45 passed / 45**</t>
+          <t>**48 passed / 48**</t>
         </is>
       </c>
     </row>
@@ -980,7 +980,7 @@
     <col width="56" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="80" customWidth="1" min="5" max="5"/>
+    <col width="61" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
@@ -1038,12 +1038,12 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>**Pending**</t>
+          <t>**Done**</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>Decision doc exists in `docs/DECISION_supervision_audit_row.md`; implementation ticket pending</t>
+          <t>Decision adopted; implemented in v294</t>
         </is>
       </c>
     </row>
@@ -1065,12 +1065,12 @@
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>**Pending**</t>
+          <t>**Done**</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Decision doc exists in `docs/DECISION_retention_holdback.md`; implementation ticket pending</t>
+          <t>Decision adopted; implemented in v294</t>
         </is>
       </c>
     </row>
@@ -1326,12 +1326,12 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>**Pending**</t>
+          <t>**Done**</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>Blocked by 1.2 decision</t>
+          <t>`projects.retention_percentage`, `retention_withheld`/`retention_released`, auto-withholding trigger</t>
         </is>
       </c>
     </row>
@@ -1353,12 +1353,12 @@
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>**Pending**</t>
+          <t>**Done**</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Blocked by 1.1 decision</t>
+          <t>`project_period_closes`, `close_project_period()` / `reopen_project_period()` RPCs</t>
         </is>
       </c>
     </row>
@@ -2003,7 +2003,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -2026,82 +2026,96 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>- `18dd0c4` — ci: Dependabot weekly npm updates</t>
+          <t>- `0e8a0ab` — fix: handle soft-deleted deposits in retention sync trigger + regenerate specs</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>- `2f93da7` — build: `npm run health` script</t>
+          <t>- `c4eadcb` — feat: v294 retention/holdback tracking + supervision period-close audit rows</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>- `edbe70d` — test: expand Utils tests (clamp, ilikeOr, sleep)</t>
+          <t>- `18dd0c4` — ci: Dependabot weekly npm updates</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>- `c138724` — test: add Auth.fromEmail and safeName unit tests</t>
+          <t>- `2f93da7` — build: `npm run health` script</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>- `682f7e1` — chore: expose App on window</t>
+          <t>- `edbe70d` — test: expand Utils tests (clamp, ilikeOr, sleep)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>- `344958a` — ci: run npm audit in CI/deploy workflows</t>
+          <t>- `c138724` — test: add Auth.fromEmail and safeName unit tests</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>- `b52eb1d` — test: expose API/Crud on window + add Crud guard tests</t>
+          <t>- `682f7e1` — chore: expose App on window</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>- `7a95736` — perf: v293 add common indexes</t>
+          <t>- `344958a` — ci: run npm audit in CI/deploy workflows</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>- `160886b` — ci: secret-scan workflow</t>
+          <t>- `b52eb1d` — test: expose API/Crud on window + add Crud guard tests</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>- `5445fb8` — docs+security: changelog v292, hardening status, pre-commit hook</t>
+          <t>- `7a95736` — perf: v293 add common indexes</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
+          <t>- `160886b` — ci: secret-scan workflow</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>- `5445fb8` — docs+security: changelog v292, hardening status, pre-commit hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
           <t>- `58968e2` — feat: v292 office_vendor_income SQL alignment + accounting unit tests</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="14">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="A9:H9"/>
@@ -2110,7 +2124,9 @@
     <mergeCell ref="A7:H7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A13:H13"/>
     <mergeCell ref="A11:H11"/>
+    <mergeCell ref="A14:H14"/>
     <mergeCell ref="A5:H5"/>
     <mergeCell ref="A8:H8"/>
     <mergeCell ref="A6:H6"/>

</xml_diff>